<commit_message>
results sensitivity tech selection CaL
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/tech_sel_CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/tech_sel_CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE65"/>
+  <dimension ref="A1:AE107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7174,6 +7174,4332 @@
       <c r="AE65" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260418214936_dh_1_ctax_250_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>11848649.15001597</v>
+      </c>
+      <c r="B66" t="n">
+        <v>4496791.901331041</v>
+      </c>
+      <c r="C66" t="n">
+        <v>3254895.4035373</v>
+      </c>
+      <c r="D66" t="n">
+        <v>3922233.632322108</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>8419025.533653149</v>
+      </c>
+      <c r="G66" t="n">
+        <v>3254895.4035373</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-2403520.371525242</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>2578248.584350757</v>
+      </c>
+      <c r="M66" t="n">
+        <v>11848649.15001597</v>
+      </c>
+      <c r="N66" t="n">
+        <v>25784.82635823538</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>25784.82635823538</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>25782.48584350741</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0</v>
+      </c>
+      <c r="S66" t="n">
+        <v>0</v>
+      </c>
+      <c r="T66" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" t="n">
+        <v>2.340514728183982</v>
+      </c>
+      <c r="V66" t="n">
+        <v>19.99300003051758</v>
+      </c>
+      <c r="W66" t="n">
+        <v>11848649.15001597</v>
+      </c>
+      <c r="X66" t="n">
+        <v>11848649.15001597</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426231215_dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>16087.92112087848</v>
+      </c>
+      <c r="I67" t="n">
+        <v>-14068696.34301499</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="n">
+        <v>21309807.07334101</v>
+      </c>
+      <c r="M67" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="N67" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" t="n">
+        <v>0</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0</v>
+      </c>
+      <c r="V67" t="n">
+        <v>17.72200012207031</v>
+      </c>
+      <c r="W67" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="X67" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426231514_dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>250352.7371741842</v>
+      </c>
+      <c r="I68" t="n">
+        <v>-21487808.21638926</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
+        <v>21418154.55076566</v>
+      </c>
+      <c r="M68" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="N68" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="R68" t="n">
+        <v>0</v>
+      </c>
+      <c r="S68" t="n">
+        <v>0</v>
+      </c>
+      <c r="T68" t="n">
+        <v>0</v>
+      </c>
+      <c r="U68" t="n">
+        <v>0</v>
+      </c>
+      <c r="V68" t="n">
+        <v>16.14400005340576</v>
+      </c>
+      <c r="W68" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="X68" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426231800_dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>871463.3829878251</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-29676874.86506916</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="n">
+        <v>21705418.22445447</v>
+      </c>
+      <c r="M69" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="N69" t="n">
+        <v>217054.1822445446</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>217054.1822445446</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>217054.1822445447</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>10.57999992370605</v>
+      </c>
+      <c r="W69" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="X69" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426232056_dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>-18630105.33902203</v>
+      </c>
+      <c r="B70" t="n">
+        <v>15743592.69407945</v>
+      </c>
+      <c r="C70" t="n">
+        <v>4455672.404650554</v>
+      </c>
+      <c r="D70" t="n">
+        <v>13314518.67751076</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>29058111.37159021</v>
+      </c>
+      <c r="G70" t="n">
+        <v>4455672.404650554</v>
+      </c>
+      <c r="H70" t="n">
+        <v>4245838.178656002</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-61063981.60668926</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
+        <v>4674254.312770459</v>
+      </c>
+      <c r="M70" t="n">
+        <v>-18630105.33902203</v>
+      </c>
+      <c r="N70" t="n">
+        <v>46747.40497228439</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>46747.40497228439</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>46742.54312770459</v>
+      </c>
+      <c r="R70" t="n">
+        <v>0</v>
+      </c>
+      <c r="S70" t="n">
+        <v>0</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0</v>
+      </c>
+      <c r="U70" t="n">
+        <v>4.861844579786982</v>
+      </c>
+      <c r="V70" t="n">
+        <v>8.682000160217285</v>
+      </c>
+      <c r="W70" t="n">
+        <v>-18630105.33902203</v>
+      </c>
+      <c r="X70" t="n">
+        <v>-18630105.33902203</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426232334_dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="B71" t="n">
+        <v>15922388.65264793</v>
+      </c>
+      <c r="C71" t="n">
+        <v>4490087.410045396</v>
+      </c>
+      <c r="D71" t="n">
+        <v>13450876.04205032</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>29373264.69469825</v>
+      </c>
+      <c r="G71" t="n">
+        <v>4490087.410045396</v>
+      </c>
+      <c r="H71" t="n">
+        <v>4563155.252214096</v>
+      </c>
+      <c r="I71" t="n">
+        <v>-74000697.31960672</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
+        <v>4661161.082765235</v>
+      </c>
+      <c r="M71" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="N71" t="n">
+        <v>46616.51447436517</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>46616.51447436517</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>46611.61082765232</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" t="n">
+        <v>0</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" t="n">
+        <v>4.903646712883647</v>
+      </c>
+      <c r="V71" t="n">
+        <v>7.629999876022339</v>
+      </c>
+      <c r="W71" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="X71" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426232616_dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="B72" t="n">
+        <v>16073837.21594865</v>
+      </c>
+      <c r="C72" t="n">
+        <v>4519238.533844642</v>
+      </c>
+      <c r="D72" t="n">
+        <v>13563156.11808991</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>29636993.33403856</v>
+      </c>
+      <c r="G72" t="n">
+        <v>4519238.533844642</v>
+      </c>
+      <c r="H72" t="n">
+        <v>4697191.196630822</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-86735147.74642958</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="n">
+        <v>4604431.358401258</v>
+      </c>
+      <c r="M72" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="N72" t="n">
+        <v>46049.24827690521</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>46049.24827690521</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>46044.31358401258</v>
+      </c>
+      <c r="R72" t="n">
+        <v>0</v>
+      </c>
+      <c r="S72" t="n">
+        <v>0</v>
+      </c>
+      <c r="T72" t="n">
+        <v>0</v>
+      </c>
+      <c r="U72" t="n">
+        <v>4.934692892651643</v>
+      </c>
+      <c r="V72" t="n">
+        <v>8.282999992370605</v>
+      </c>
+      <c r="W72" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="X72" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426232903_dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="B73" t="n">
+        <v>16196872.91946809</v>
+      </c>
+      <c r="C73" t="n">
+        <v>4542920.693297691</v>
+      </c>
+      <c r="D73" t="n">
+        <v>13652363.65409414</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
+        <v>29849236.57356223</v>
+      </c>
+      <c r="G73" t="n">
+        <v>4542920.693297691</v>
+      </c>
+      <c r="H73" t="n">
+        <v>4741325.92959027</v>
+      </c>
+      <c r="I73" t="n">
+        <v>-99355790.54539734</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" t="n">
+        <v>4538794.319774911</v>
+      </c>
+      <c r="M73" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="N73" t="n">
+        <v>45392.900392944</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>45392.900392944</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>45387.9431977491</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0</v>
+      </c>
+      <c r="S73" t="n">
+        <v>0</v>
+      </c>
+      <c r="T73" t="n">
+        <v>0</v>
+      </c>
+      <c r="U73" t="n">
+        <v>4.957195194896266</v>
+      </c>
+      <c r="V73" t="n">
+        <v>7.963000059127808</v>
+      </c>
+      <c r="W73" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="X73" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426233202_dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>13040862.50238379</v>
+      </c>
+      <c r="B74" t="n">
+        <v>4606697.01508003</v>
+      </c>
+      <c r="C74" t="n">
+        <v>3296311.782785068</v>
+      </c>
+      <c r="D74" t="n">
+        <v>3997918.753663895</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>8604615.768743925</v>
+      </c>
+      <c r="G74" t="n">
+        <v>3296311.782785068</v>
+      </c>
+      <c r="H74" t="n">
+        <v>61649.7985881268</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-2341213.361767607</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="n">
+        <v>3419498.514034281</v>
+      </c>
+      <c r="M74" t="n">
+        <v>13040862.50238379</v>
+      </c>
+      <c r="N74" t="n">
+        <v>22799.03816194926</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>22799.03816194926</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>22796.65676022858</v>
+      </c>
+      <c r="R74" t="n">
+        <v>0</v>
+      </c>
+      <c r="S74" t="n">
+        <v>0</v>
+      </c>
+      <c r="T74" t="n">
+        <v>0</v>
+      </c>
+      <c r="U74" t="n">
+        <v>2.381401720705843</v>
+      </c>
+      <c r="V74" t="n">
+        <v>22.9850001335144</v>
+      </c>
+      <c r="W74" t="n">
+        <v>13040862.50238379</v>
+      </c>
+      <c r="X74" t="n">
+        <v>13040862.50238379</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426233509_dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>10690839.24273433</v>
+      </c>
+      <c r="B75" t="n">
+        <v>4566176.867306454</v>
+      </c>
+      <c r="C75" t="n">
+        <v>3281042.319004511</v>
+      </c>
+      <c r="D75" t="n">
+        <v>3973447.188271914</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>8539624.055578368</v>
+      </c>
+      <c r="G75" t="n">
+        <v>3281042.319004511</v>
+      </c>
+      <c r="H75" t="n">
+        <v>71057.05106035013</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-4737273.459144993</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>3536389.276236092</v>
+      </c>
+      <c r="M75" t="n">
+        <v>10690839.24273433</v>
+      </c>
+      <c r="N75" t="n">
+        <v>23578.30071292132</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>23578.30071292132</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>23575.92850824055</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0</v>
+      </c>
+      <c r="S75" t="n">
+        <v>0</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0</v>
+      </c>
+      <c r="U75" t="n">
+        <v>2.372204680639244</v>
+      </c>
+      <c r="V75" t="n">
+        <v>39.32699990272522</v>
+      </c>
+      <c r="W75" t="n">
+        <v>10690839.24273433</v>
+      </c>
+      <c r="X75" t="n">
+        <v>10690839.24273433</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426233740_dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>13212651.19193472</v>
+      </c>
+      <c r="B76" t="n">
+        <v>4470200.639116395</v>
+      </c>
+      <c r="C76" t="n">
+        <v>3244873.974516834</v>
+      </c>
+      <c r="D76" t="n">
+        <v>5265215.841826544</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" t="n">
+        <v>9735416.480942938</v>
+      </c>
+      <c r="G76" t="n">
+        <v>3244873.974516834</v>
+      </c>
+      <c r="H76" t="n">
+        <v>-4.494150224729545e-16</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-2423590.327672481</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>2655951.064147431</v>
+      </c>
+      <c r="M76" t="n">
+        <v>13212651.19193472</v>
+      </c>
+      <c r="N76" t="n">
+        <v>26561.8414433927</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>26561.8414433927</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>26559.51064147439</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0</v>
+      </c>
+      <c r="U76" t="n">
+        <v>2.330801918209394</v>
+      </c>
+      <c r="V76" t="n">
+        <v>19.79200005531311</v>
+      </c>
+      <c r="W76" t="n">
+        <v>13212651.19193472</v>
+      </c>
+      <c r="X76" t="n">
+        <v>13212651.19193472</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426234609_dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="B77" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>16087.92112087848</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-14068696.34301499</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
+        <v>21309807.07334101</v>
+      </c>
+      <c r="M77" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="N77" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>213098.07073341</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0</v>
+      </c>
+      <c r="V77" t="n">
+        <v>14.46800017356873</v>
+      </c>
+      <c r="W77" t="n">
+        <v>7692927.423242348</v>
+      </c>
+      <c r="X77" t="n">
+        <v>7692927.423242366</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>1.769512891769409e-08</v>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426234908_dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="B78" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>250352.7371741842</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-21487808.21638926</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>21418154.55076566</v>
+      </c>
+      <c r="M78" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="N78" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>214181.5455076566</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0</v>
+      </c>
+      <c r="V78" t="n">
+        <v>13.62000012397766</v>
+      </c>
+      <c r="W78" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="X78" t="n">
+        <v>616427.8433460556</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426235150_dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="B79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>435728.7717954639</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>871463.3829878251</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-29676874.86506916</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>21705418.22445447</v>
+      </c>
+      <c r="M79" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="N79" t="n">
+        <v>217054.1822445446</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>217054.1822445446</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>217054.1822445447</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0</v>
+      </c>
+      <c r="V79" t="n">
+        <v>8.826000213623047</v>
+      </c>
+      <c r="W79" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="X79" t="n">
+        <v>-6664264.485831395</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426235443_dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>-18630105.33902204</v>
+      </c>
+      <c r="B80" t="n">
+        <v>15743592.69407944</v>
+      </c>
+      <c r="C80" t="n">
+        <v>4455672.404650554</v>
+      </c>
+      <c r="D80" t="n">
+        <v>13314518.67751076</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="n">
+        <v>29058111.3715902</v>
+      </c>
+      <c r="G80" t="n">
+        <v>4455672.404650554</v>
+      </c>
+      <c r="H80" t="n">
+        <v>4245838.178656002</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-61063981.60668926</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>4674254.312770459</v>
+      </c>
+      <c r="M80" t="n">
+        <v>-18630105.33902204</v>
+      </c>
+      <c r="N80" t="n">
+        <v>46747.40497228439</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>46747.40497228439</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>46742.54312770459</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" t="n">
+        <v>0</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0</v>
+      </c>
+      <c r="U80" t="n">
+        <v>4.861844579786982</v>
+      </c>
+      <c r="V80" t="n">
+        <v>8.700000047683716</v>
+      </c>
+      <c r="W80" t="n">
+        <v>-18630105.33902204</v>
+      </c>
+      <c r="X80" t="n">
+        <v>-18630105.33902204</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260426235720_dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="B81" t="n">
+        <v>15922388.65264793</v>
+      </c>
+      <c r="C81" t="n">
+        <v>4490087.410045397</v>
+      </c>
+      <c r="D81" t="n">
+        <v>13450876.04205032</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>29373264.69469825</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4490087.410045397</v>
+      </c>
+      <c r="H81" t="n">
+        <v>4563155.252214096</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-74000697.31960672</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>4661161.082765235</v>
+      </c>
+      <c r="M81" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="N81" t="n">
+        <v>46616.51447436516</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>46616.51447436516</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>46611.61082765232</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0</v>
+      </c>
+      <c r="U81" t="n">
+        <v>4.903646712883647</v>
+      </c>
+      <c r="V81" t="n">
+        <v>8.35099983215332</v>
+      </c>
+      <c r="W81" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="X81" t="n">
+        <v>-30913028.87988374</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427000003_dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="B82" t="n">
+        <v>16073837.21594865</v>
+      </c>
+      <c r="C82" t="n">
+        <v>4519238.533844642</v>
+      </c>
+      <c r="D82" t="n">
+        <v>13563156.11808991</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>29636993.33403856</v>
+      </c>
+      <c r="G82" t="n">
+        <v>4519238.533844642</v>
+      </c>
+      <c r="H82" t="n">
+        <v>4697191.196630822</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-86735147.74642958</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
+        <v>4604431.358401258</v>
+      </c>
+      <c r="M82" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="N82" t="n">
+        <v>46049.24827690521</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="n">
+        <v>46049.24827690521</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>46044.31358401258</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" t="n">
+        <v>0</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0</v>
+      </c>
+      <c r="U82" t="n">
+        <v>4.934692892651643</v>
+      </c>
+      <c r="V82" t="n">
+        <v>7.988000154495239</v>
+      </c>
+      <c r="W82" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="X82" t="n">
+        <v>-43277293.3235143</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE82" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427000250_dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="B83" t="n">
+        <v>16196872.91946809</v>
+      </c>
+      <c r="C83" t="n">
+        <v>4542920.693297691</v>
+      </c>
+      <c r="D83" t="n">
+        <v>13652363.65409414</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>29849236.57356223</v>
+      </c>
+      <c r="G83" t="n">
+        <v>4542920.693297691</v>
+      </c>
+      <c r="H83" t="n">
+        <v>4741325.92959027</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-99355790.54539734</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
+        <v>4538794.319774911</v>
+      </c>
+      <c r="M83" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="N83" t="n">
+        <v>45392.900392944</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="n">
+        <v>45392.900392944</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>45387.9431977491</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0</v>
+      </c>
+      <c r="S83" t="n">
+        <v>0</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" t="n">
+        <v>4.957195194896266</v>
+      </c>
+      <c r="V83" t="n">
+        <v>8.628999948501587</v>
+      </c>
+      <c r="W83" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="X83" t="n">
+        <v>-55683513.02917224</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE83" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427000546_dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>14431071.78964609</v>
+      </c>
+      <c r="B84" t="n">
+        <v>4597296.63512145</v>
+      </c>
+      <c r="C84" t="n">
+        <v>3292769.37810029</v>
+      </c>
+      <c r="D84" t="n">
+        <v>5381978.745640699</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>9979275.380762149</v>
+      </c>
+      <c r="G84" t="n">
+        <v>3292769.37810029</v>
+      </c>
+      <c r="H84" t="n">
+        <v>61649.7985881268</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-2345211.372792644</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
+        <v>3442588.60498817</v>
+      </c>
+      <c r="M84" t="n">
+        <v>14431071.78964609</v>
+      </c>
+      <c r="N84" t="n">
+        <v>22952.97017746751</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" t="n">
+        <v>22952.97017746751</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>22950.59069992109</v>
+      </c>
+      <c r="R84" t="n">
+        <v>0</v>
+      </c>
+      <c r="S84" t="n">
+        <v>0</v>
+      </c>
+      <c r="T84" t="n">
+        <v>0</v>
+      </c>
+      <c r="U84" t="n">
+        <v>2.379477546459687</v>
+      </c>
+      <c r="V84" t="n">
+        <v>24.27699995040894</v>
+      </c>
+      <c r="W84" t="n">
+        <v>14431071.78964609</v>
+      </c>
+      <c r="X84" t="n">
+        <v>14431071.78964609</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427000853_dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>12074880.56187627</v>
+      </c>
+      <c r="B85" t="n">
+        <v>4547623.293883766</v>
+      </c>
+      <c r="C85" t="n">
+        <v>3274050.516632522</v>
+      </c>
+      <c r="D85" t="n">
+        <v>5344290.869430327</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>9891914.163314093</v>
+      </c>
+      <c r="G85" t="n">
+        <v>3274050.516632522</v>
+      </c>
+      <c r="H85" t="n">
+        <v>71036.38152518011</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-4757860.047339633</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>3595739.547744107</v>
+      </c>
+      <c r="M85" t="n">
+        <v>12074880.56187627</v>
+      </c>
+      <c r="N85" t="n">
+        <v>23973.96424259028</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>23973.96424259028</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>23971.59698496072</v>
+      </c>
+      <c r="R85" t="n">
+        <v>0</v>
+      </c>
+      <c r="S85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T85" t="n">
+        <v>0</v>
+      </c>
+      <c r="U85" t="n">
+        <v>2.36725762972274</v>
+      </c>
+      <c r="V85" t="n">
+        <v>39.24499988555908</v>
+      </c>
+      <c r="W85" t="n">
+        <v>12074880.56187627</v>
+      </c>
+      <c r="X85" t="n">
+        <v>12074880.56187627</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC85" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE85" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427001123_dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>7287157.798800359</v>
+      </c>
+      <c r="B86" t="n">
+        <v>15710707.40302627</v>
+      </c>
+      <c r="C86" t="n">
+        <v>4449342.577745812</v>
+      </c>
+      <c r="D86" t="n">
+        <v>13288983.33702855</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>28999690.74005482</v>
+      </c>
+      <c r="G86" t="n">
+        <v>4449342.577745812</v>
+      </c>
+      <c r="H86" t="n">
+        <v>2688168.814440039</v>
+      </c>
+      <c r="I86" t="n">
+        <v>-34828433.70764709</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
+        <v>5978389.374206769</v>
+      </c>
+      <c r="M86" t="n">
+        <v>7287157.798800359</v>
+      </c>
+      <c r="N86" t="n">
+        <v>39860.78270039293</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="n">
+        <v>39860.78270039293</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>39855.92916137846</v>
+      </c>
+      <c r="R86" t="n">
+        <v>0</v>
+      </c>
+      <c r="S86" t="n">
+        <v>0</v>
+      </c>
+      <c r="T86" t="n">
+        <v>0</v>
+      </c>
+      <c r="U86" t="n">
+        <v>4.853539014477754</v>
+      </c>
+      <c r="V86" t="n">
+        <v>33.32500004768372</v>
+      </c>
+      <c r="W86" t="n">
+        <v>7287157.798800359</v>
+      </c>
+      <c r="X86" t="n">
+        <v>7287157.798800359</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE86" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427001513_dh_0.5_ctax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>-4433725.727619075</v>
+      </c>
+      <c r="B87" t="n">
+        <v>15893509.93144037</v>
+      </c>
+      <c r="C87" t="n">
+        <v>4484528.775755719</v>
+      </c>
+      <c r="D87" t="n">
+        <v>13429145.40202023</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>29322655.3334606</v>
+      </c>
+      <c r="G87" t="n">
+        <v>4484528.775755719</v>
+      </c>
+      <c r="H87" t="n">
+        <v>3100383.637032812</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-47354685.83597761</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>6013392.362109399</v>
+      </c>
+      <c r="M87" t="n">
+        <v>-4433725.727619075</v>
+      </c>
+      <c r="N87" t="n">
+        <v>40094.17970646705</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="n">
+        <v>40094.17970646705</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>40089.28241406269</v>
+      </c>
+      <c r="R87" t="n">
+        <v>0</v>
+      </c>
+      <c r="S87" t="n">
+        <v>0</v>
+      </c>
+      <c r="T87" t="n">
+        <v>0</v>
+      </c>
+      <c r="U87" t="n">
+        <v>4.897292404390106</v>
+      </c>
+      <c r="V87" t="n">
+        <v>20.55000019073486</v>
+      </c>
+      <c r="W87" t="n">
+        <v>-4433725.727619075</v>
+      </c>
+      <c r="X87" t="n">
+        <v>-4433725.727619075</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE87" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427001755_dh_0.5_ctax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>-16414487.48231448</v>
+      </c>
+      <c r="B88" t="n">
+        <v>16050311.04193305</v>
+      </c>
+      <c r="C88" t="n">
+        <v>4514710.168594393</v>
+      </c>
+      <c r="D88" t="n">
+        <v>13545891.95604631</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>29596202.99797937</v>
+      </c>
+      <c r="G88" t="n">
+        <v>4514710.168594393</v>
+      </c>
+      <c r="H88" t="n">
+        <v>3782854.452765602</v>
+      </c>
+      <c r="I88" t="n">
+        <v>-60606865.29221875</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>6298610.19056492</v>
+      </c>
+      <c r="M88" t="n">
+        <v>-16414487.48231448</v>
+      </c>
+      <c r="N88" t="n">
+        <v>41995.6647143538</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" t="n">
+        <v>41995.6647143538</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>41990.73460376615</v>
+      </c>
+      <c r="R88" t="n">
+        <v>0</v>
+      </c>
+      <c r="S88" t="n">
+        <v>0</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0</v>
+      </c>
+      <c r="U88" t="n">
+        <v>4.930110587670076</v>
+      </c>
+      <c r="V88" t="n">
+        <v>11.14300012588501</v>
+      </c>
+      <c r="W88" t="n">
+        <v>-16414487.48231448</v>
+      </c>
+      <c r="X88" t="n">
+        <v>-16414487.48231448</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE88" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427002025_dh_0.5_ctax_150_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>-28652772.37601389</v>
+      </c>
+      <c r="B89" t="n">
+        <v>16174836.49502872</v>
+      </c>
+      <c r="C89" t="n">
+        <v>4538679.078039516</v>
+      </c>
+      <c r="D89" t="n">
+        <v>13636513.07924368</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>29811349.57427239</v>
+      </c>
+      <c r="G89" t="n">
+        <v>4538679.078039516</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4356865.402324745</v>
+      </c>
+      <c r="I89" t="n">
+        <v>-73923269.5859455</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>6563603.155294962</v>
+      </c>
+      <c r="M89" t="n">
+        <v>-28652772.37601389</v>
+      </c>
+      <c r="N89" t="n">
+        <v>43762.30770555997</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="n">
+        <v>43762.30770555997</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>43757.35436863308</v>
+      </c>
+      <c r="R89" t="n">
+        <v>0</v>
+      </c>
+      <c r="S89" t="n">
+        <v>0</v>
+      </c>
+      <c r="T89" t="n">
+        <v>0</v>
+      </c>
+      <c r="U89" t="n">
+        <v>4.953336926892972</v>
+      </c>
+      <c r="V89" t="n">
+        <v>9.974999904632568</v>
+      </c>
+      <c r="W89" t="n">
+        <v>-28652772.37601389</v>
+      </c>
+      <c r="X89" t="n">
+        <v>-28652772.37601389</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE89" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427002405_dh_0.5_ctax_150_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>-41022586.62006754</v>
+      </c>
+      <c r="B90" t="n">
+        <v>16293057.31453755</v>
+      </c>
+      <c r="C90" t="n">
+        <v>4561434.458942718</v>
+      </c>
+      <c r="D90" t="n">
+        <v>13720931.10355682</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>30013988.41809437</v>
+      </c>
+      <c r="G90" t="n">
+        <v>4561434.458942718</v>
+      </c>
+      <c r="H90" t="n">
+        <v>4606156.101975969</v>
+      </c>
+      <c r="I90" t="n">
+        <v>-86826778.13297923</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
+        <v>6622612.533898629</v>
+      </c>
+      <c r="M90" t="n">
+        <v>-41022586.62006754</v>
+      </c>
+      <c r="N90" t="n">
+        <v>44155.72342611813</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="n">
+        <v>44155.72342611813</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>44150.75022599086</v>
+      </c>
+      <c r="R90" t="n">
+        <v>0</v>
+      </c>
+      <c r="S90" t="n">
+        <v>0</v>
+      </c>
+      <c r="T90" t="n">
+        <v>0</v>
+      </c>
+      <c r="U90" t="n">
+        <v>4.973200127307342</v>
+      </c>
+      <c r="V90" t="n">
+        <v>11.69600009918213</v>
+      </c>
+      <c r="W90" t="n">
+        <v>-41022586.62006754</v>
+      </c>
+      <c r="X90" t="n">
+        <v>-41022586.62006754</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC90" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427002624_dh_0.5_ctax_150_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>-53448129.73973404</v>
+      </c>
+      <c r="B91" t="n">
+        <v>16401593.92028187</v>
+      </c>
+      <c r="C91" t="n">
+        <v>4582325.802920148</v>
+      </c>
+      <c r="D91" t="n">
+        <v>13797360.08969022</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>30198954.0099721</v>
+      </c>
+      <c r="G91" t="n">
+        <v>4582325.802920148</v>
+      </c>
+      <c r="H91" t="n">
+        <v>4722926.495495129</v>
+      </c>
+      <c r="I91" t="n">
+        <v>-99559696.98394628</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>6607360.935824871</v>
+      </c>
+      <c r="M91" t="n">
+        <v>-53448129.73973404</v>
+      </c>
+      <c r="N91" t="n">
+        <v>44054.06288743335</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>44054.06288743335</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>44049.07290549911</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0</v>
+      </c>
+      <c r="S91" t="n">
+        <v>0</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0</v>
+      </c>
+      <c r="U91" t="n">
+        <v>4.98998193424757</v>
+      </c>
+      <c r="V91" t="n">
+        <v>9.716000080108643</v>
+      </c>
+      <c r="W91" t="n">
+        <v>-53448129.73973404</v>
+      </c>
+      <c r="X91" t="n">
+        <v>-53448129.73973404</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427003019_dh_0.5_ctax_150_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>15560833.01007283</v>
+      </c>
+      <c r="B92" t="n">
+        <v>4638797.828254792</v>
+      </c>
+      <c r="C92" t="n">
+        <v>3308409.86350393</v>
+      </c>
+      <c r="D92" t="n">
+        <v>5410189.842212491</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>10048987.67046728</v>
+      </c>
+      <c r="G92" t="n">
+        <v>3308409.86350393</v>
+      </c>
+      <c r="H92" t="n">
+        <v>61660.43239431651</v>
+      </c>
+      <c r="I92" t="n">
+        <v>-2329868.57703856</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>4471643.620745858</v>
+      </c>
+      <c r="M92" t="n">
+        <v>15560833.01007283</v>
+      </c>
+      <c r="N92" t="n">
+        <v>22360.60498654781</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>22360.60498654781</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>22358.21810372924</v>
+      </c>
+      <c r="R92" t="n">
+        <v>0</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0</v>
+      </c>
+      <c r="T92" t="n">
+        <v>0</v>
+      </c>
+      <c r="U92" t="n">
+        <v>2.386882818679005</v>
+      </c>
+      <c r="V92" t="n">
+        <v>27.55100011825562</v>
+      </c>
+      <c r="W92" t="n">
+        <v>15560833.01007283</v>
+      </c>
+      <c r="X92" t="n">
+        <v>15560833.01007283</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC92" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE92" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427003238_dh_0.5_ctax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>13228328.6145497</v>
+      </c>
+      <c r="B93" t="n">
+        <v>4620853.653073619</v>
+      </c>
+      <c r="C93" t="n">
+        <v>3301647.09165551</v>
+      </c>
+      <c r="D93" t="n">
+        <v>5398398.024687304</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>10019251.67776092</v>
+      </c>
+      <c r="G93" t="n">
+        <v>3301647.09165551</v>
+      </c>
+      <c r="H93" t="n">
+        <v>61650.59590798803</v>
+      </c>
+      <c r="I93" t="n">
+        <v>-4671525.521148329</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>4517304.770373608</v>
+      </c>
+      <c r="M93" t="n">
+        <v>13228328.6145497</v>
+      </c>
+      <c r="N93" t="n">
+        <v>22588.90788029622</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>22588.90788029622</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>22586.52385186816</v>
+      </c>
+      <c r="R93" t="n">
+        <v>0</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" t="n">
+        <v>2.384028428155403</v>
+      </c>
+      <c r="V93" t="n">
+        <v>44.68099999427795</v>
+      </c>
+      <c r="W93" t="n">
+        <v>13228328.6145497</v>
+      </c>
+      <c r="X93" t="n">
+        <v>13228328.6145497</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE93" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427003514_dh_0.5_ctax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>9202100.071973849</v>
+      </c>
+      <c r="B94" t="n">
+        <v>16019060.67144454</v>
+      </c>
+      <c r="C94" t="n">
+        <v>4508695.034485301</v>
+      </c>
+      <c r="D94" t="n">
+        <v>13522850.91777706</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
+        <v>29541911.5892216</v>
+      </c>
+      <c r="G94" t="n">
+        <v>4508695.034485301</v>
+      </c>
+      <c r="H94" t="n">
+        <v>2673165.140720346</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-34941033.33542764</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>7419361.642974245</v>
+      </c>
+      <c r="M94" t="n">
+        <v>9202100.071973849</v>
+      </c>
+      <c r="N94" t="n">
+        <v>37101.73209153737</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>37101.73209153737</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>37096.80821487122</v>
+      </c>
+      <c r="R94" t="n">
+        <v>0</v>
+      </c>
+      <c r="S94" t="n">
+        <v>0</v>
+      </c>
+      <c r="T94" t="n">
+        <v>0</v>
+      </c>
+      <c r="U94" t="n">
+        <v>4.923876666152148</v>
+      </c>
+      <c r="V94" t="n">
+        <v>32.92499995231628</v>
+      </c>
+      <c r="W94" t="n">
+        <v>9202100.071973849</v>
+      </c>
+      <c r="X94" t="n">
+        <v>9202100.071973849</v>
+      </c>
+      <c r="Y94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE94" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427003809_dh_0.5_ctax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>-2507756.240945558</v>
+      </c>
+      <c r="B95" t="n">
+        <v>16150007.75034616</v>
+      </c>
+      <c r="C95" t="n">
+        <v>4533899.99136978</v>
+      </c>
+      <c r="D95" t="n">
+        <v>13618580.12901534</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="n">
+        <v>29768587.8793615</v>
+      </c>
+      <c r="G95" t="n">
+        <v>4533899.99136978</v>
+      </c>
+      <c r="H95" t="n">
+        <v>2912259.440196565</v>
+      </c>
+      <c r="I95" t="n">
+        <v>-47171726.54230385</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>7449222.990430449</v>
+      </c>
+      <c r="M95" t="n">
+        <v>-2507756.240945558</v>
+      </c>
+      <c r="N95" t="n">
+        <v>37251.06384184915</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>37251.06384184915</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>37246.11495215222</v>
+      </c>
+      <c r="R95" t="n">
+        <v>0</v>
+      </c>
+      <c r="S95" t="n">
+        <v>0</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0</v>
+      </c>
+      <c r="U95" t="n">
+        <v>4.948889696932932</v>
+      </c>
+      <c r="V95" t="n">
+        <v>27.80799984931946</v>
+      </c>
+      <c r="W95" t="n">
+        <v>-2507756.240945558</v>
+      </c>
+      <c r="X95" t="n">
+        <v>-2507756.240945558</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427004246_dh_0.5_ctax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>-14400748.50100967</v>
+      </c>
+      <c r="B96" t="n">
+        <v>16265050.4721611</v>
+      </c>
+      <c r="C96" t="n">
+        <v>4556043.645642489</v>
+      </c>
+      <c r="D96" t="n">
+        <v>13701049.47671651</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="n">
+        <v>29966099.94887761</v>
+      </c>
+      <c r="G96" t="n">
+        <v>4556043.645642489</v>
+      </c>
+      <c r="H96" t="n">
+        <v>3402887.343609172</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-60077680.5802563</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>7751901.141117349</v>
+      </c>
+      <c r="M96" t="n">
+        <v>-14400748.50100967</v>
+      </c>
+      <c r="N96" t="n">
+        <v>38764.47435884221</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>38764.47435884221</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>38759.50570558672</v>
+      </c>
+      <c r="R96" t="n">
+        <v>0</v>
+      </c>
+      <c r="S96" t="n">
+        <v>0</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0</v>
+      </c>
+      <c r="U96" t="n">
+        <v>4.968653255496437</v>
+      </c>
+      <c r="V96" t="n">
+        <v>19.87299990653992</v>
+      </c>
+      <c r="W96" t="n">
+        <v>-14400748.50100967</v>
+      </c>
+      <c r="X96" t="n">
+        <v>-14400748.50100967</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427004524_dh_0.5_ctax_200_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>-26530279.59724355</v>
+      </c>
+      <c r="B97" t="n">
+        <v>16383168.58989547</v>
+      </c>
+      <c r="C97" t="n">
+        <v>4578779.258301765</v>
+      </c>
+      <c r="D97" t="n">
+        <v>13784458.56541067</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="n">
+        <v>30167627.15530615</v>
+      </c>
+      <c r="G97" t="n">
+        <v>4578779.258301765</v>
+      </c>
+      <c r="H97" t="n">
+        <v>4023262.714944505</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-73483604.98745266</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>8183656.261656694</v>
+      </c>
+      <c r="M97" t="n">
+        <v>-26530279.59724355</v>
+      </c>
+      <c r="N97" t="n">
+        <v>40923.26854040816</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" t="n">
+        <v>40923.26854040816</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>40918.28130828348</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0</v>
+      </c>
+      <c r="U97" t="n">
+        <v>4.987232124698783</v>
+      </c>
+      <c r="V97" t="n">
+        <v>16.61199998855591</v>
+      </c>
+      <c r="W97" t="n">
+        <v>-26530279.59724355</v>
+      </c>
+      <c r="X97" t="n">
+        <v>-26530279.59724355</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE97" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427004754_dh_0.5_ctax_200_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>-38857321.87619775</v>
+      </c>
+      <c r="B98" t="n">
+        <v>16458619.19692968</v>
+      </c>
+      <c r="C98" t="n">
+        <v>4593302.142761324</v>
+      </c>
+      <c r="D98" t="n">
+        <v>13837028.55108122</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" t="n">
+        <v>30295647.7480109</v>
+      </c>
+      <c r="G98" t="n">
+        <v>4593302.142761324</v>
+      </c>
+      <c r="H98" t="n">
+        <v>4456762.345405993</v>
+      </c>
+      <c r="I98" t="n">
+        <v>-86704261.24992996</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="n">
+        <v>8501227.137553997</v>
+      </c>
+      <c r="M98" t="n">
+        <v>-38857321.87619775</v>
+      </c>
+      <c r="N98" t="n">
+        <v>42511.13382676578</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" t="n">
+        <v>42511.13382676578</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>42506.13568776999</v>
+      </c>
+      <c r="R98" t="n">
+        <v>0</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0</v>
+      </c>
+      <c r="U98" t="n">
+        <v>4.998138995807191</v>
+      </c>
+      <c r="V98" t="n">
+        <v>14.21499991416931</v>
+      </c>
+      <c r="W98" t="n">
+        <v>-38857321.87619775</v>
+      </c>
+      <c r="X98" t="n">
+        <v>-38857321.87619775</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE98" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427005022_dh_0.5_ctax_200_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>-51273773.25995292</v>
+      </c>
+      <c r="B99" t="n">
+        <v>16524372.73269592</v>
+      </c>
+      <c r="C99" t="n">
+        <v>4605958.51545701</v>
+      </c>
+      <c r="D99" t="n">
+        <v>13882329.64163589</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>30406702.37433181</v>
+      </c>
+      <c r="G99" t="n">
+        <v>4605958.51545701</v>
+      </c>
+      <c r="H99" t="n">
+        <v>4628408.545349183</v>
+      </c>
+      <c r="I99" t="n">
+        <v>-99507455.33460274</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
+        <v>8592612.639511822</v>
+      </c>
+      <c r="M99" t="n">
+        <v>-51273773.25995292</v>
+      </c>
+      <c r="N99" t="n">
+        <v>42968.07014759087</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="n">
+        <v>42968.07014759087</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>42963.06319755909</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0</v>
+      </c>
+      <c r="U99" t="n">
+        <v>5.006950031788233</v>
+      </c>
+      <c r="V99" t="n">
+        <v>13.93899989128113</v>
+      </c>
+      <c r="W99" t="n">
+        <v>-51273773.25995292</v>
+      </c>
+      <c r="X99" t="n">
+        <v>-51273773.25995292</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427005505_dh_0.5_ctax_200_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>16672197.28829921</v>
+      </c>
+      <c r="B100" t="n">
+        <v>4661718.814893891</v>
+      </c>
+      <c r="C100" t="n">
+        <v>3317048.040521846</v>
+      </c>
+      <c r="D100" t="n">
+        <v>5424399.573123281</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="n">
+        <v>10086118.38801717</v>
+      </c>
+      <c r="G100" t="n">
+        <v>3317048.040521846</v>
+      </c>
+      <c r="H100" t="n">
+        <v>61666.56126501279</v>
+      </c>
+      <c r="I100" t="n">
+        <v>-2323878.543375981</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>5531242.841871162</v>
+      </c>
+      <c r="M100" t="n">
+        <v>16672197.28829921</v>
+      </c>
+      <c r="N100" t="n">
+        <v>22127.36116624189</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" t="n">
+        <v>22127.36116624189</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>22124.9713674846</v>
+      </c>
+      <c r="R100" t="n">
+        <v>0</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0</v>
+      </c>
+      <c r="U100" t="n">
+        <v>2.389798757207401</v>
+      </c>
+      <c r="V100" t="n">
+        <v>31.23000001907349</v>
+      </c>
+      <c r="W100" t="n">
+        <v>16672197.28829921</v>
+      </c>
+      <c r="X100" t="n">
+        <v>16672197.28829921</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE100" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427005731_dh_0.5_ctax_250_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>14347211.39145043</v>
+      </c>
+      <c r="B101" t="n">
+        <v>4651290.989729667</v>
+      </c>
+      <c r="C101" t="n">
+        <v>3313118.018564924</v>
+      </c>
+      <c r="D101" t="n">
+        <v>5418043.277904866</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" t="n">
+        <v>10069334.26763453</v>
+      </c>
+      <c r="G101" t="n">
+        <v>3313118.018564924</v>
+      </c>
+      <c r="H101" t="n">
+        <v>61666.5612650128</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-4652828.267591804</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>5555920.811577762</v>
+      </c>
+      <c r="M101" t="n">
+        <v>14347211.39145043</v>
+      </c>
+      <c r="N101" t="n">
+        <v>22226.07181116975</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
+        <v>22226.07181116975</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>22223.68324631104</v>
+      </c>
+      <c r="R101" t="n">
+        <v>0</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0</v>
+      </c>
+      <c r="T101" t="n">
+        <v>0</v>
+      </c>
+      <c r="U101" t="n">
+        <v>2.38856485872207</v>
+      </c>
+      <c r="V101" t="n">
+        <v>31.99599981307983</v>
+      </c>
+      <c r="W101" t="n">
+        <v>14347211.39145043</v>
+      </c>
+      <c r="X101" t="n">
+        <v>14347211.39145043</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE101" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427010016_dh_0.5_ctax_250_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>11016511.95139173</v>
+      </c>
+      <c r="B102" t="n">
+        <v>16232978.38752413</v>
+      </c>
+      <c r="C102" t="n">
+        <v>4549870.346342875</v>
+      </c>
+      <c r="D102" t="n">
+        <v>13678205.69976766</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="n">
+        <v>29911184.08729179</v>
+      </c>
+      <c r="G102" t="n">
+        <v>4549870.346342875</v>
+      </c>
+      <c r="H102" t="n">
+        <v>2680106.341195275</v>
+      </c>
+      <c r="I102" t="n">
+        <v>-35029575.42615055</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
+        <v>8904926.602712339</v>
+      </c>
+      <c r="M102" t="n">
+        <v>11016511.95139173</v>
+      </c>
+      <c r="N102" t="n">
+        <v>35624.66975391798</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="n">
+        <v>35624.66975391798</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>35619.70641084936</v>
+      </c>
+      <c r="R102" t="n">
+        <v>0</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
+      <c r="T102" t="n">
+        <v>0</v>
+      </c>
+      <c r="U102" t="n">
+        <v>4.963343068617274</v>
+      </c>
+      <c r="V102" t="n">
+        <v>31.56299996376038</v>
+      </c>
+      <c r="W102" t="n">
+        <v>11016511.95139173</v>
+      </c>
+      <c r="X102" t="n">
+        <v>11016511.95139173</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427010301_dh_0.5_ctax_250_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>-692234.180535946</v>
+      </c>
+      <c r="B103" t="n">
+        <v>16358017.18949536</v>
+      </c>
+      <c r="C103" t="n">
+        <v>4573938.066211139</v>
+      </c>
+      <c r="D103" t="n">
+        <v>13766802.45616681</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>30124819.64566217</v>
+      </c>
+      <c r="G103" t="n">
+        <v>4573938.066211139</v>
+      </c>
+      <c r="H103" t="n">
+        <v>2798027.498950305</v>
+      </c>
+      <c r="I103" t="n">
+        <v>-47038378.26025783</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
+        <v>8849358.868898269</v>
+      </c>
+      <c r="M103" t="n">
+        <v>-692234.180535946</v>
+      </c>
+      <c r="N103" t="n">
+        <v>35402.41889322743</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" t="n">
+        <v>35402.41889322743</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>35397.43547559308</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0</v>
+      </c>
+      <c r="T103" t="n">
+        <v>0</v>
+      </c>
+      <c r="U103" t="n">
+        <v>4.983417634350486</v>
+      </c>
+      <c r="V103" t="n">
+        <v>26.33599996566772</v>
+      </c>
+      <c r="W103" t="n">
+        <v>-692234.180535946</v>
+      </c>
+      <c r="X103" t="n">
+        <v>-692234.180535946</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427010546_dh_0.5_ctax_250_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>-12530696.99333975</v>
+      </c>
+      <c r="B104" t="n">
+        <v>16441372.71287405</v>
+      </c>
+      <c r="C104" t="n">
+        <v>4589982.504853573</v>
+      </c>
+      <c r="D104" t="n">
+        <v>13825074.11821725</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="n">
+        <v>30266446.8310913</v>
+      </c>
+      <c r="G104" t="n">
+        <v>4589982.504853573</v>
+      </c>
+      <c r="H104" t="n">
+        <v>3110135.421657719</v>
+      </c>
+      <c r="I104" t="n">
+        <v>-59589789.62064991</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
+        <v>9092527.869707562</v>
+      </c>
+      <c r="M104" t="n">
+        <v>-12530696.99333975</v>
+      </c>
+      <c r="N104" t="n">
+        <v>36375.10720870664</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" t="n">
+        <v>36375.10720870664</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>36370.11147883026</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0</v>
+      </c>
+      <c r="T104" t="n">
+        <v>0</v>
+      </c>
+      <c r="U104" t="n">
+        <v>4.995729876408505</v>
+      </c>
+      <c r="V104" t="n">
+        <v>22.36700010299683</v>
+      </c>
+      <c r="W104" t="n">
+        <v>-12530696.99333975</v>
+      </c>
+      <c r="X104" t="n">
+        <v>-12530696.99333975</v>
+      </c>
+      <c r="Y104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427011116_dh_0.5_ctax_250_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>-24552622.4736787</v>
+      </c>
+      <c r="B105" t="n">
+        <v>16512671.00474571</v>
+      </c>
+      <c r="C105" t="n">
+        <v>4603706.143346588</v>
+      </c>
+      <c r="D105" t="n">
+        <v>13874303.53677997</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="n">
+        <v>30386974.54152568</v>
+      </c>
+      <c r="G105" t="n">
+        <v>4603706.143346588</v>
+      </c>
+      <c r="H105" t="n">
+        <v>3605761.813966109</v>
+      </c>
+      <c r="I105" t="n">
+        <v>-72721922.11417568</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="n">
+        <v>9572857.141658606</v>
+      </c>
+      <c r="M105" t="n">
+        <v>-24552622.4736787</v>
+      </c>
+      <c r="N105" t="n">
+        <v>38296.4339971544</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>38296.4339971544</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>38291.42856663443</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0</v>
+      </c>
+      <c r="T105" t="n">
+        <v>0</v>
+      </c>
+      <c r="U105" t="n">
+        <v>5.005430519991434</v>
+      </c>
+      <c r="V105" t="n">
+        <v>20.61100006103516</v>
+      </c>
+      <c r="W105" t="n">
+        <v>-24552622.4736787</v>
+      </c>
+      <c r="X105" t="n">
+        <v>-24552622.4736787</v>
+      </c>
+      <c r="Y105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC105" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427011354_dh_0.5_ctax_250_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>-36777785.01047975</v>
+      </c>
+      <c r="B106" t="n">
+        <v>16565573.66809903</v>
+      </c>
+      <c r="C106" t="n">
+        <v>4613888.954296472</v>
+      </c>
+      <c r="D106" t="n">
+        <v>13910450.25564022</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>30476023.92373925</v>
+      </c>
+      <c r="G106" t="n">
+        <v>4613888.954296472</v>
+      </c>
+      <c r="H106" t="n">
+        <v>4196364.934509845</v>
+      </c>
+      <c r="I106" t="n">
+        <v>-86255927.01569271</v>
+      </c>
+      <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
+        <v>10191864.19266739</v>
+      </c>
+      <c r="M106" t="n">
+        <v>-36777785.01047975</v>
+      </c>
+      <c r="N106" t="n">
+        <v>40772.46888292589</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" t="n">
+        <v>40772.46888292589</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>40767.45677066955</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0</v>
+      </c>
+      <c r="S106" t="n">
+        <v>0</v>
+      </c>
+      <c r="T106" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" t="n">
+        <v>5.012112256361405</v>
+      </c>
+      <c r="V106" t="n">
+        <v>18.71300005912781</v>
+      </c>
+      <c r="W106" t="n">
+        <v>-36777785.01047975</v>
+      </c>
+      <c r="X106" t="n">
+        <v>-36777785.01047975</v>
+      </c>
+      <c r="Y106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC106" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427011631_dh_0.5_ctax_250_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>-49150093.59491254</v>
+      </c>
+      <c r="B107" t="n">
+        <v>16615813.79475743</v>
+      </c>
+      <c r="C107" t="n">
+        <v>4623559.27483296</v>
+      </c>
+      <c r="D107" t="n">
+        <v>13944485.43966322</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>30560299.23442065</v>
+      </c>
+      <c r="G107" t="n">
+        <v>4623559.27483296</v>
+      </c>
+      <c r="H107" t="n">
+        <v>4507780.577357303</v>
+      </c>
+      <c r="I107" t="n">
+        <v>-99336792.851096</v>
+      </c>
+      <c r="J107" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
+        <v>10495060.16957255</v>
+      </c>
+      <c r="M107" t="n">
+        <v>-49150093.59491254</v>
+      </c>
+      <c r="N107" t="n">
+        <v>41985.25874012785</v>
+      </c>
+      <c r="O107" t="n">
+        <v>0</v>
+      </c>
+      <c r="P107" t="n">
+        <v>41985.25874012785</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>41980.2406782902</v>
+      </c>
+      <c r="R107" t="n">
+        <v>0</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+      <c r="T107" t="n">
+        <v>0</v>
+      </c>
+      <c r="U107" t="n">
+        <v>5.018061837674999</v>
+      </c>
+      <c r="V107" t="n">
+        <v>17.79900002479553</v>
+      </c>
+      <c r="W107" t="n">
+        <v>-49150093.59491254</v>
+      </c>
+      <c r="X107" t="n">
+        <v>-49150093.59491254</v>
+      </c>
+      <c r="Y107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC107" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\tech_sel_CaL\20260427011905_dh_0.5_ctax_250_el_price_400</t>
         </is>
       </c>
     </row>

</xml_diff>